<commit_message>
Round 1 paper revision updates.
</commit_message>
<xml_diff>
--- a/output/psa_results/psa_descriptive_table1_edited.xlsx
+++ b/output/psa_results/psa_descriptive_table1_edited.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29328"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\RDobs\Downloads\Graduate School\gangestad_dobson\prolific1_gangestad\output\results\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\RDobs\Downloads\Graduate School\gangestad_dobson\prolific1_gangestad\psa_manuscript\output\psa_results\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{2DC72EE3-4581-47EC-AFA5-4A86248499FC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D26D848A-E551-4E4B-B92A-1446458A65E3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-27840" yWindow="960" windowWidth="21600" windowHeight="11235" xr2:uid="{03FBB896-CCCF-4955-8FC6-69347AF6C6FB}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{03FBB896-CCCF-4955-8FC6-69347AF6C6FB}"/>
   </bookViews>
   <sheets>
     <sheet name="descriptive_table1" sheetId="1" r:id="rId1"/>
@@ -163,7 +163,40 @@
     <t>Descriptive statistics by study</t>
   </si>
   <si>
-    <t>Note.</t>
+    <r>
+      <t xml:space="preserve">Note. Age and relationship length values are M </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>(</t>
+    </r>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>SD</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>)</t>
+    </r>
   </si>
 </sst>
 </file>

</xml_diff>